<commit_message>
feat(P4): README and Artifacts Update.
</commit_message>
<xml_diff>
--- a/04-ai-governance-and-technical-lifecycle/artifacts/A-01_AI_Use_Case_Inventory.xlsx
+++ b/04-ai-governance-and-technical-lifecycle/artifacts/A-01_AI_Use_Case_Inventory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Career\Portfolio\Project4\Artifacts V2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rityshree\my_project\04-ai-governance-and-technical-lifecycle\artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288A509D-6FAD-4206-BBB6-718A70B22839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89E675F7-6BCB-40E2-89BE-151B949386C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -361,9 +361,6 @@
     <t>~2.5M historical credit application records (7 years); ~300K loan performance sequences</t>
   </si>
   <si>
-    <t>AWS Bedrock + SageMaker: NCL-AWS-PROD-002</t>
-  </si>
-  <si>
     <t>Core Banking Engine, Credit Bureau Gateway, Loan Origination System (LOS), Underwriter Portal</t>
   </si>
   <si>
@@ -665,6 +662,9 @@
   </si>
   <si>
     <t>Approval History</t>
+  </si>
+  <si>
+    <t>AWS Bedrock + SageMaker: NCL-AWS-PILOT-002 (scenario environment identifier)</t>
   </si>
 </sst>
 </file>
@@ -981,7 +981,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1029,12 +1029,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="14" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1062,14 +1056,6 @@
     <xf numFmtId="0" fontId="13" fillId="14" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1101,7 +1087,12 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1421,7 +1412,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1446,7 +1437,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.3">
@@ -1550,66 +1541,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="24.6" x14ac:dyDescent="0.4">
-      <c r="A1" s="43" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" s="45" customFormat="1" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+      <c r="A1" s="37" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="44" t="s">
+      <c r="C3" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="D3" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="44" t="s">
+      <c r="E3" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="44" t="s">
+      <c r="F3" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="44" t="s">
+      <c r="G3" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="44" t="s">
+      <c r="H3" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="44" t="s">
+      <c r="I3" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="44" t="s">
+      <c r="J3" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="44" t="s">
+      <c r="K3" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="44" t="s">
+      <c r="L3" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="M3" s="44" t="s">
+      <c r="M3" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="N3" s="44" t="s">
+      <c r="N3" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="O3" s="44" t="s">
+      <c r="O3" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="P3" s="44" t="s">
+      <c r="P3" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="Q3" s="44" t="s">
+      <c r="Q3" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="R3" s="44" t="s">
+      <c r="R3" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="S3" s="44" t="s">
+      <c r="S3" s="38" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1618,7 +1609,7 @@
         <v>32</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>55</v>
@@ -1677,7 +1668,7 @@
         <v>33</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>72</v>
@@ -1698,7 +1689,7 @@
         <v>36</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J5" s="8" t="s">
         <v>77</v>
@@ -1736,7 +1727,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>84</v>
@@ -1795,7 +1786,7 @@
         <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>98</v>
@@ -1831,22 +1822,22 @@
         <v>107</v>
       </c>
       <c r="N7" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="O7" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="P7" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="P7" s="8" t="s">
+      <c r="Q7" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="R7" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="S7" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="S7" s="8" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1857,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2C49DF5-7D0E-4769-A8B7-7E9C90A30A86}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" style="18" customWidth="1"/>
@@ -1868,126 +1859,120 @@
     <col min="7" max="16384" width="8.88671875" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+    </row>
+    <row r="2" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-    </row>
-    <row r="2" spans="1:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-    </row>
-    <row r="3" spans="1:7" s="22" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3" s="29" t="s">
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+    </row>
+    <row r="3" spans="1:6" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="B3" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="C3" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="D3" s="27" t="s">
         <v>146</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="E3" s="27" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="F3" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="24" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="B4" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="C4" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="D4" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="E4" s="22" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="F4" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B5" s="26" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="B5" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="C5" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="D5" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="E5" s="24" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="F5" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="B6" s="24" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="B6" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="C6" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="D6" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="E6" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="22" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="26" t="s">
+    <row r="7" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="B7" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="C7" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="D7" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="E7" s="24" t="s">
         <v>122</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2019,305 +2004,305 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
+      <c r="A1" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:10" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-    </row>
-    <row r="3" spans="1:10" s="22" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="A2" s="40"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+    </row>
+    <row r="3" spans="1:10" s="20" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="28" t="s">
+        <v>191</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="J4" s="31" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="33" t="s">
+        <v>195</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="J5" s="34" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="37.799999999999997" x14ac:dyDescent="0.3">
+      <c r="A6" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>199</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="I6" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="J6" s="31" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="37.799999999999997" x14ac:dyDescent="0.3">
+      <c r="A7" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>203</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>166</v>
+      </c>
+      <c r="G7" s="36" t="s">
+        <v>206</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>207</v>
+      </c>
+      <c r="J7" s="34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="C3" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="F3" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="G3" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="H3" s="21" t="s">
-        <v>157</v>
-      </c>
-      <c r="I3" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="J3" s="21" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="35" t="s">
-        <v>190</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>191</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="36" t="s">
+      <c r="C8" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="34" t="s">
-        <v>192</v>
-      </c>
-      <c r="I4" s="35" t="s">
-        <v>193</v>
-      </c>
-      <c r="J4" s="37" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="33" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="C5" s="38" t="s">
-        <v>195</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>196</v>
-      </c>
-      <c r="F5" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="36" t="s">
+      <c r="H8" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="I8" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="J8" s="31" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="G9" s="36" t="s">
+        <v>174</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="I9" s="32" t="s">
+        <v>176</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>178</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="F10" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="G10" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="39" t="s">
-        <v>194</v>
-      </c>
-      <c r="I5" s="38" t="s">
-        <v>197</v>
-      </c>
-      <c r="J5" s="40" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A6" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="35" t="s">
-        <v>199</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>200</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>202</v>
-      </c>
-      <c r="I6" s="35" t="s">
-        <v>203</v>
-      </c>
-      <c r="J6" s="37" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="37.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="38" t="s">
-        <v>204</v>
-      </c>
-      <c r="C7" s="38" t="s">
-        <v>205</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="F7" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="G7" s="42" t="s">
-        <v>207</v>
-      </c>
-      <c r="H7" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="I7" s="38" t="s">
-        <v>208</v>
-      </c>
-      <c r="J7" s="40" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
+      <c r="H10" s="28" t="s">
+        <v>181</v>
+      </c>
+      <c r="I10" s="29" t="s">
+        <v>182</v>
+      </c>
+      <c r="J10" s="31" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="35" t="s">
-        <v>164</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>165</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>166</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>167</v>
-      </c>
-      <c r="G8" s="36" t="s">
+      <c r="B11" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" s="33" t="s">
+        <v>183</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="G11" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="34" t="s">
-        <v>168</v>
-      </c>
-      <c r="I8" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="J8" s="37" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="C9" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="D9" s="38" t="s">
-        <v>172</v>
-      </c>
-      <c r="E9" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="G9" s="42" t="s">
-        <v>175</v>
-      </c>
-      <c r="H9" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="I9" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="J9" s="40" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>164</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>179</v>
-      </c>
-      <c r="D10" s="35" t="s">
-        <v>180</v>
-      </c>
-      <c r="E10" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="F10" s="35" t="s">
-        <v>174</v>
-      </c>
-      <c r="G10" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="I10" s="35" t="s">
-        <v>183</v>
-      </c>
-      <c r="J10" s="37" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="38" t="s">
-        <v>164</v>
-      </c>
-      <c r="C11" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="D11" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="F11" s="38" t="s">
+      <c r="H11" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="G11" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="39" t="s">
+      <c r="I11" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="I11" s="38" t="s">
+      <c r="J11" s="34" t="s">
         <v>188</v>
-      </c>
-      <c r="J11" s="40" t="s">
-        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>